<commit_message>
Update site from notebooks
</commit_message>
<xml_diff>
--- a/codespace/DetroitRiverCase/results/ch3_fw3_concordant_lda_random_split_cv_confusion_matrix.xlsx
+++ b/codespace/DetroitRiverCase/results/ch3_fw3_concordant_lda_random_split_cv_confusion_matrix.xlsx
@@ -458,17 +458,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1.40 +/- 0.02</t>
+          <t>1.89 +/- 0.02</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1.47 +/- 0.02</t>
+          <t>3.73 +/- 0.03</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.13 +/- 0.01</t>
+          <t>1.38 +/- 0.02</t>
         </is>
       </c>
     </row>
@@ -480,17 +480,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.27 +/- 0.02</t>
+          <t>2.03 +/- 0.01</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>7.72 +/- 0.02</t>
+          <t>7.07 +/- 0.01</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.00 +/- 0.00</t>
+          <t>0.90 +/- 0.01</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.27 +/- 0.02</t>
+          <t>0.11 +/- 0.01</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.46 +/- 0.02</t>
+          <t>1.60 +/- 0.02</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.27 +/- 0.02</t>
+          <t>6.29 +/- 0.02</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>85% +/- 0% (n = 17)</t>
+          <t>61% +/- 0% (n = 25)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>

</xml_diff>